<commit_message>
Fix roxygen documentation issues, and excel date
</commit_message>
<xml_diff>
--- a/data-raw/parametra_template.xlsx
+++ b/data-raw/parametra_template.xlsx
@@ -15,24 +15,24 @@
     <sheet name="ControlPlan" sheetId="89" state="visible" r:id="rId7"/>
     <sheet name="CostBiosecurity" sheetId="90" state="visible" r:id="rId8"/>
     <sheet name="OtherRelevantInformation" sheetId="91" state="visible" r:id="rId9"/>
-    <sheet name="LOT" sheetId="123" state="visible" r:id="rId10"/>
-    <sheet name="transmission" sheetId="124" state="visible" r:id="rId11"/>
-    <sheet name="infectious_latent_incuba_period" sheetId="125" state="visible" r:id="rId12"/>
-    <sheet name="pathogen_survival" sheetId="126" state="visible" r:id="rId13"/>
-    <sheet name="diagnostic_test" sheetId="127" state="visible" r:id="rId14"/>
-    <sheet name="within_herd_prevalence" sheetId="128" state="visible" r:id="rId15"/>
-    <sheet name="regional_prevalence" sheetId="129" state="visible" r:id="rId16"/>
-    <sheet name="control_plan" sheetId="130" state="visible" r:id="rId17"/>
-    <sheet name="cost_biosecurity" sheetId="131" state="visible" r:id="rId18"/>
-    <sheet name="other" sheetId="132" state="visible" r:id="rId19"/>
-    <sheet name="Crossref" sheetId="133" state="visible" r:id="rId20"/>
+    <sheet name="LOT" sheetId="156" state="visible" r:id="rId10"/>
+    <sheet name="transmission" sheetId="157" state="visible" r:id="rId11"/>
+    <sheet name="infectious_latent_incuba_period" sheetId="158" state="visible" r:id="rId12"/>
+    <sheet name="pathogen_survival" sheetId="159" state="visible" r:id="rId13"/>
+    <sheet name="diagnostic_test" sheetId="160" state="visible" r:id="rId14"/>
+    <sheet name="within_herd_prevalence" sheetId="161" state="visible" r:id="rId15"/>
+    <sheet name="regional_prevalence" sheetId="162" state="visible" r:id="rId16"/>
+    <sheet name="control_plan" sheetId="163" state="visible" r:id="rId17"/>
+    <sheet name="cost_biosecurity" sheetId="164" state="visible" r:id="rId18"/>
+    <sheet name="other" sheetId="165" state="visible" r:id="rId19"/>
+    <sheet name="Crossref" sheetId="166" state="visible" r:id="rId20"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="594">
   <si>
     <t>Use this workbook to submit new PARAMETRA records.</t>
   </si>
@@ -1893,6 +1893,15 @@
   </si>
   <si>
     <t xml:space="preserve">Last update:2026-06-29 19:20:25 CEST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last update:30/06/2026 09:34:58 CEST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last update:30/06/2026 09:36:01 CEST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last update:30/06/2026 09:36:28 CEST</t>
   </si>
 </sst>
 </file>
@@ -2290,7 +2299,7 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
Pre-release meeting review (added last_accessed date for costs table), changed "url_check_failed" to "url_manual_check"
</commit_message>
<xml_diff>
--- a/data-raw/parametra_template.xlsx
+++ b/data-raw/parametra_template.xlsx
@@ -15,24 +15,24 @@
     <sheet name="ControlPlan" sheetId="89" state="visible" r:id="rId7"/>
     <sheet name="CostBiosecurity" sheetId="90" state="visible" r:id="rId8"/>
     <sheet name="OtherRelevantInformation" sheetId="91" state="visible" r:id="rId9"/>
-    <sheet name="LOT" sheetId="156" state="visible" r:id="rId10"/>
-    <sheet name="transmission" sheetId="157" state="visible" r:id="rId11"/>
-    <sheet name="infectious_latent_incuba_period" sheetId="158" state="visible" r:id="rId12"/>
-    <sheet name="pathogen_survival" sheetId="159" state="visible" r:id="rId13"/>
-    <sheet name="diagnostic_test" sheetId="160" state="visible" r:id="rId14"/>
-    <sheet name="within_herd_prevalence" sheetId="161" state="visible" r:id="rId15"/>
-    <sheet name="regional_prevalence" sheetId="162" state="visible" r:id="rId16"/>
-    <sheet name="control_plan" sheetId="163" state="visible" r:id="rId17"/>
-    <sheet name="cost_biosecurity" sheetId="164" state="visible" r:id="rId18"/>
-    <sheet name="other" sheetId="165" state="visible" r:id="rId19"/>
-    <sheet name="Crossref" sheetId="166" state="visible" r:id="rId20"/>
+    <sheet name="LOT" sheetId="167" state="visible" r:id="rId10"/>
+    <sheet name="transmission" sheetId="168" state="visible" r:id="rId11"/>
+    <sheet name="infectious_latent_incuba_period" sheetId="169" state="visible" r:id="rId12"/>
+    <sheet name="pathogen_survival" sheetId="170" state="visible" r:id="rId13"/>
+    <sheet name="diagnostic_test" sheetId="171" state="visible" r:id="rId14"/>
+    <sheet name="within_herd_prevalence" sheetId="172" state="visible" r:id="rId15"/>
+    <sheet name="regional_prevalence" sheetId="173" state="visible" r:id="rId16"/>
+    <sheet name="control_plan" sheetId="174" state="visible" r:id="rId17"/>
+    <sheet name="cost_biosecurity" sheetId="175" state="visible" r:id="rId18"/>
+    <sheet name="other" sheetId="176" state="visible" r:id="rId19"/>
+    <sheet name="Crossref" sheetId="177" state="visible" r:id="rId20"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="594">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="597">
   <si>
     <t>Use this workbook to submit new PARAMETRA records.</t>
   </si>
@@ -1902,6 +1902,15 @@
   </si>
   <si>
     <t xml:space="preserve">Last update:30/06/2026 09:36:28 CEST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last update:14/07/2026 13:46:16 CEST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">url_manual_check</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URL check done manually. Automatic URL check failed or returned an unexpected status (rate limited, server error, access restricted...).</t>
   </si>
 </sst>
 </file>
@@ -2299,7 +2308,7 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>3</v>
@@ -3973,10 +3982,10 @@
         <v>356</v>
       </c>
       <c r="B149" t="s">
-        <v>544</v>
+        <v>595</v>
       </c>
       <c r="C149" t="s">
-        <v>545</v>
+        <v>596</v>
       </c>
     </row>
     <row r="150">

</xml_diff>